<commit_message>
Refactor reporting bot into expense-based workflow
</commit_message>
<xml_diff>
--- a/Templates/Example.xlsx
+++ b/Templates/Example.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Yakov\Рабочий стол\PROGRAMMIROVANIE\Python\A5\grant_report_helper\Templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Yakov\Рабочий стол\PROGRAMMIROVANIE\Python\A5\grant_report2\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEA57EC0-9357-475D-9488-2C549220F863}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13063623-FAF5-4DF5-AC5A-84D4902FBA90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1515" yWindow="1515" windowWidth="21600" windowHeight="11190" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -75,56 +75,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C1" authorId="0" shapeId="0" xr:uid="{D7E87FF7-FB65-43EE-A7A1-A82DA86DA74E}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>Yakov Mokin:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-Короткое название категорий (обязательный столбец)</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{9C372BCD-97DC-4489-A345-2E6C3764A924}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>Yakov Mokin:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-Короткое название статьи расходов. Должен быть для каждой статьи расходов
-(обязательный столбец)</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{FEC12CC9-8272-49E1-B2B0-4F484941839C}">
+    <comment ref="C1" authorId="0" shapeId="0" xr:uid="{FEC12CC9-8272-49E1-B2B0-4F484941839C}">
       <text>
         <r>
           <rPr>
@@ -153,7 +104,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
   <si>
     <t>Категория</t>
   </si>
@@ -161,117 +112,60 @@
     <t>Статья Расходов</t>
   </si>
   <si>
-    <t>Категория_Short</t>
-  </si>
-  <si>
-    <t>Статья Расходов_Short</t>
-  </si>
-  <si>
     <t>Бюджет</t>
   </si>
   <si>
     <t>Канцелярия и расходные материалы</t>
   </si>
   <si>
-    <t>КАНЦ</t>
-  </si>
-  <si>
     <t>Полиграфическая продукция</t>
   </si>
   <si>
     <t>Изготовление брендированной продукции</t>
   </si>
   <si>
-    <t>ПОЛИГРАФ</t>
-  </si>
-  <si>
-    <t>бренд</t>
-  </si>
-  <si>
     <t>Подарки и сувенирная продукция</t>
   </si>
   <si>
     <t>Научно-популярные книги, 20 шт</t>
   </si>
   <si>
-    <t>ПОДАР</t>
-  </si>
-  <si>
-    <t>книг</t>
-  </si>
-  <si>
     <t>Проживание и питание</t>
   </si>
   <si>
     <t>Продукты питания и товары для организации кофе-брейков</t>
   </si>
   <si>
-    <t>ПРиПИТ</t>
-  </si>
-  <si>
-    <t>кофебрейк</t>
-  </si>
-  <si>
     <t>Услуги по доставке воды</t>
   </si>
   <si>
-    <t>вода</t>
-  </si>
-  <si>
     <t>Аренда помещений</t>
   </si>
   <si>
-    <t>АРЕНД</t>
-  </si>
-  <si>
     <t>Закупка оборудования</t>
   </si>
   <si>
-    <t>ОБОРУД</t>
-  </si>
-  <si>
     <t>Дополнительные услуги и товары для проекта</t>
   </si>
   <si>
-    <t>ДОПУСЛ</t>
-  </si>
-  <si>
     <t>Расходы на ПО</t>
   </si>
   <si>
-    <t>ПО</t>
-  </si>
-  <si>
     <t>Сайт и приложение</t>
   </si>
   <si>
-    <t>САЙТ</t>
-  </si>
-  <si>
     <t>Расходы на связь</t>
   </si>
   <si>
-    <t>СВЯЗЬ</t>
-  </si>
-  <si>
     <t>Транспортные расходы</t>
   </si>
   <si>
-    <t>ТРАНСП</t>
-  </si>
-  <si>
     <t>Аренда оборудования</t>
   </si>
   <si>
-    <t>АРОБОРУД</t>
-  </si>
-  <si>
     <t>Информационные услуги</t>
   </si>
   <si>
-    <t>ИНФУСЛ</t>
-  </si>
-  <si>
     <t>Канцелярские товары для уроков</t>
   </si>
   <si>
@@ -279,15 +173,6 @@
   </si>
   <si>
     <t>Покупка принтера</t>
-  </si>
-  <si>
-    <t>зал</t>
-  </si>
-  <si>
-    <t>принт</t>
-  </si>
-  <si>
-    <t>канц</t>
   </si>
 </sst>
 </file>
@@ -592,236 +477,160 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E15"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="4" width="27" style="1" customWidth="1"/>
+    <col min="1" max="2" width="27" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+    </row>
+    <row r="2" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="B2" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" s="4">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+      <c r="B3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C2" s="4" t="s">
+      <c r="C3" s="4">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E2" s="4">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
+      <c r="B4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="C4" s="4">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="B5" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="C5" s="4">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="4">
+      <c r="C6" s="4">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="4">
         <v>10000</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="4" t="s">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="B8" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" s="4">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="B9" s="4"/>
+      <c r="C9" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="4">
-        <v>20000</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
+      <c r="B10" s="4"/>
+      <c r="C10" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B11" s="4"/>
+      <c r="C11" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="B12" s="4"/>
+      <c r="C12" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="B13" s="4"/>
+      <c r="C13" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="E5" s="4">
-        <v>5000</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" s="4" t="s">
+      <c r="B14" s="4"/>
+      <c r="C14" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E6" s="4">
-        <v>2000</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="E7" s="4">
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="E8" s="4">
-        <v>12000</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A9" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B9" s="4"/>
-      <c r="C9" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D10" s="4"/>
-      <c r="E10" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B11" s="4"/>
-      <c r="C11" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B12" s="4"/>
-      <c r="C12" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="B13" s="4"/>
-      <c r="C13" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="B14" s="4"/>
-      <c r="C14" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" s="4" t="s">
-        <v>37</v>
-      </c>
       <c r="B15" s="4"/>
-      <c r="C15" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="D15" s="4"/>
-      <c r="E15" s="4">
+      <c r="C15" s="4">
         <v>0</v>
       </c>
     </row>

</xml_diff>